<commit_message>
feat(import): quitter-only alumni, open current units, nameless rows and surname photos (#816)
- A Quitters row on no year sheet imports as an alumnus of the year it left
  in, from its join day (else the year's start) to its leave day; every
  listed date form reads; an override line can place a row in a year; a row
  with no usable date is listed by row as an unclear quitter.
- The override input is one file, overrides.csv (kind,sheet,row,value), for
  seat handovers and quitter years; it replaces handovers.csv.
- Units the current sheet names and the database lacks are created open; the
  report lists every unit to create by name, open or closed.
- Sheet rows with no first and no last name are skipped, never matched.
- Photos: <id>-<surname> is always a people_rows.csv id; a surname-only file
  matches the one advisor with that surname (CSV or workbook advisor row).
- README, fake fixtures and tests cover each rule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/import/fixtures/rules/roster.xlsx
+++ b/scripts/import/fixtures/rules/roster.xlsx
@@ -181,6 +181,24 @@
     <t>Hybrid Motors</t>
   </si>
   <si>
+    <t>Rosa</t>
+  </si>
+  <si>
+    <t>Sarti</t>
+  </si>
+  <si>
+    <t>rosa.sarti@example.com</t>
+  </si>
+  <si>
+    <t>Avionics (AVI)</t>
+  </si>
+  <si>
+    <t>Flight Software (FSW)</t>
+  </si>
+  <si>
+    <t>name.surname@studenti.example.com</t>
+  </si>
+  <si>
     <t>Number</t>
   </si>
   <si>
@@ -308,6 +326,81 @@
   </si>
   <si>
     <t>Left the Team on:</t>
+  </si>
+  <si>
+    <t>Joined the Team on:</t>
+  </si>
+  <si>
+    <t>10/11/2021</t>
+  </si>
+  <si>
+    <t>Sergio</t>
+  </si>
+  <si>
+    <t>Tosi</t>
+  </si>
+  <si>
+    <t>sergio.tosi@example.com</t>
+  </si>
+  <si>
+    <t>5/3/2024</t>
+  </si>
+  <si>
+    <t>Teresa</t>
+  </si>
+  <si>
+    <t>Ugolini</t>
+  </si>
+  <si>
+    <t>teresa.ugolini@example.com</t>
+  </si>
+  <si>
+    <t>Propulsion (PRP)</t>
+  </si>
+  <si>
+    <t>30.06.2022</t>
+  </si>
+  <si>
+    <t>Ugo</t>
+  </si>
+  <si>
+    <t>Valli</t>
+  </si>
+  <si>
+    <t>ugo.valli@example.com</t>
+  </si>
+  <si>
+    <t>Vera</t>
+  </si>
+  <si>
+    <t>Zanni</t>
+  </si>
+  <si>
+    <t>vera.zanni@example.com</t>
+  </si>
+  <si>
+    <t>Management</t>
+  </si>
+  <si>
+    <t>Walter</t>
+  </si>
+  <si>
+    <t>Bassi</t>
+  </si>
+  <si>
+    <t>walter.bassi@example.com</t>
+  </si>
+  <si>
+    <t>sometime in 2023</t>
+  </si>
+  <si>
+    <t>Xenia</t>
+  </si>
+  <si>
+    <t>Conti</t>
+  </si>
+  <si>
+    <t>xenia.conti@example.com</t>
   </si>
   <si>
     <t>Injectors (INJ)</t>
@@ -596,6 +689,58 @@
         <v>28</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" t="s">
+        <v>55</v>
+      </c>
+      <c r="M8" t="s">
+        <v>56</v>
+      </c>
+      <c r="N8" t="s">
+        <v>57</v>
+      </c>
+      <c r="P8" t="s">
+        <v>47</v>
+      </c>
+      <c r="R8" t="s">
+        <v>26</v>
+      </c>
+      <c r="S8" t="s">
+        <v>27</v>
+      </c>
+      <c r="T8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" t="s">
+        <v>58</v>
+      </c>
+      <c r="R9" t="s">
+        <v>26</v>
+      </c>
+      <c r="S9" t="s">
+        <v>27</v>
+      </c>
+      <c r="T9" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -605,7 +750,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -617,25 +762,25 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="F1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="G1" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="H1" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="I1" t="s">
         <v>12</v>
       </c>
       <c r="J1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="K1" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2">
@@ -643,19 +788,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E2" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="I2" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="J2" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3">
@@ -672,7 +817,7 @@
         <v>50</v>
       </c>
       <c r="H3" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J3" t="s">
         <v>47</v>
@@ -683,19 +828,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E4" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="H4" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="I4" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="J4" t="s">
         <v>47</v>
@@ -706,13 +851,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="E5" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="J5" t="s">
         <v>47</v>
@@ -727,7 +872,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -739,25 +884,25 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="F1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="G1" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="H1" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="I1" t="s">
         <v>12</v>
       </c>
       <c r="J1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="K1" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2">
@@ -765,19 +910,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="E2" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="H2" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="J2" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3">
@@ -785,13 +930,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C3" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E3" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="J3" t="s">
         <v>47</v>
@@ -802,16 +947,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C4" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E4" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="H4" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="J4" t="s">
         <v>47</v>
@@ -822,19 +967,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E5" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="H5" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="I5" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="J5" t="s">
         <v>47</v>
@@ -849,7 +994,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -861,25 +1006,25 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="F1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="G1" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="H1" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="I1" t="s">
         <v>12</v>
       </c>
       <c r="J1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="K1" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2">
@@ -887,19 +1032,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="H2" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="J2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3">
@@ -907,16 +1052,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C3" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E3" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="H3" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="J3" t="s">
         <v>47</v>
@@ -927,16 +1072,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C4" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E4" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="H4" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="J4" t="s">
         <v>47</v>
@@ -951,44 +1096,184 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
-        <v>54</v>
-      </c>
       <c r="E1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F1" t="s">
+        <v>63</v>
+      </c>
+      <c r="G1" t="s">
         <v>12</v>
       </c>
-      <c r="G1" t="s">
-        <v>58</v>
+      <c r="H1" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
         <v>44742</v>
       </c>
-      <c r="B2" t="s">
-        <v>92</v>
-      </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D2" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="E2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>44972</v>
+      </c>
+      <c r="B3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E3" t="s">
+        <v>106</v>
+      </c>
+      <c r="F3" t="s">
+        <v>95</v>
+      </c>
+      <c r="H3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D4" t="s">
+        <v>109</v>
+      </c>
+      <c r="E4" t="s">
+        <v>110</v>
+      </c>
+      <c r="F4" t="s">
+        <v>111</v>
+      </c>
+      <c r="G4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" s="1">
+        <v>44119</v>
+      </c>
+      <c r="C5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D5" t="s">
+        <v>114</v>
+      </c>
+      <c r="E5" t="s">
+        <v>115</v>
+      </c>
+      <c r="F5" t="s">
+        <v>97</v>
+      </c>
+      <c r="H5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6" t="s">
+        <v>116</v>
+      </c>
+      <c r="D6" t="s">
+        <v>117</v>
+      </c>
+      <c r="E6" t="s">
+        <v>118</v>
+      </c>
+      <c r="F6" t="s">
+        <v>119</v>
+      </c>
+      <c r="H6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D7" t="s">
+        <v>121</v>
+      </c>
+      <c r="E7" t="s">
+        <v>122</v>
+      </c>
+      <c r="F7" t="s">
+        <v>119</v>
+      </c>
+      <c r="H7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>123</v>
+      </c>
+      <c r="C8" t="s">
+        <v>124</v>
+      </c>
+      <c r="D8" t="s">
+        <v>125</v>
+      </c>
+      <c r="E8" t="s">
+        <v>126</v>
+      </c>
+      <c r="F8" t="s">
+        <v>119</v>
+      </c>
+      <c r="H8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1">
+        <v>45047</v>
+      </c>
+      <c r="E9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" t="s">
+        <v>95</v>
+      </c>
+      <c r="H9" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1007,7 +1292,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D1" t="s">
         <v>12</v>
@@ -1016,21 +1301,21 @@
         <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D2" t="s">
-        <v>96</v>
+        <v>127</v>
       </c>
       <c r="F2" t="s">
         <v>47</v>
@@ -1051,7 +1336,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D1" t="s">
         <v>12</v>
@@ -1060,18 +1345,18 @@
         <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="F2" t="s">
         <v>47</v>

</xml_diff>

<commit_message>
fix(import): skip Roles 22-23, read the 2022-2023 "A" and joining-day columns, keep handover givers on the team (#816)
- Roles 22-23 is not read; the 2022-2023 sheet reads its "A" column as
  Division and "Date of joining" as that year's role start.
- A seat's earlier holder whose handed-over seat was their only role gets
  an active "Member" role; a head seat in a department the run creates
  can be handed over.
- An Excel serial too large for any day reads as no day instead of
  throwing.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/import/fixtures/rules/roster.xlsx
+++ b/scripts/import/fixtures/rules/roster.xlsx
@@ -199,6 +199,27 @@
     <t>name.surname@studenti.example.com</t>
   </si>
   <si>
+    <t>Yara</t>
+  </si>
+  <si>
+    <t>Gori</t>
+  </si>
+  <si>
+    <t>yara.gori@example.com</t>
+  </si>
+  <si>
+    <t>Head of Department</t>
+  </si>
+  <si>
+    <t>Leo</t>
+  </si>
+  <si>
+    <t>Pini</t>
+  </si>
+  <si>
+    <t>leo.pini@example.com</t>
+  </si>
+  <si>
     <t>Number</t>
   </si>
   <si>
@@ -262,6 +283,12 @@
     <t>quinto.rossi@example.com</t>
   </si>
   <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Date of joining</t>
+  </si>
+  <si>
     <t>Lia</t>
   </si>
   <si>
@@ -283,6 +310,12 @@
     <t>mario.lodi@example.com</t>
   </si>
   <si>
+    <t>Liquid Propulsion</t>
+  </si>
+  <si>
+    <t>Injectors (INJ)</t>
+  </si>
+  <si>
     <t>Nora</t>
   </si>
   <si>
@@ -295,9 +328,15 @@
     <t>Vittorio Emanuele II (VES) - Management</t>
   </si>
   <si>
+    <t>1/12/2022</t>
+  </si>
+  <si>
     <t>Solid Motors</t>
   </si>
   <si>
+    <t>after the exams</t>
+  </si>
+  <si>
     <t>Oscar</t>
   </si>
   <si>
@@ -313,9 +352,6 @@
     <t>President &amp; Chief Engineer</t>
   </si>
   <si>
-    <t>Liquid Propulsion</t>
-  </si>
-  <si>
     <t>Pia</t>
   </si>
   <si>
@@ -403,7 +439,13 @@
     <t>xenia.conti@example.com</t>
   </si>
   <si>
-    <t>Injectors (INJ)</t>
+    <t>Hydraulics (HYD)</t>
+  </si>
+  <si>
+    <t>Nobody</t>
+  </si>
+  <si>
+    <t>Known</t>
   </si>
 </sst>
 </file>
@@ -741,6 +783,64 @@
         <v>28</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" t="s">
+        <v>60</v>
+      </c>
+      <c r="E10" t="s">
+        <v>61</v>
+      </c>
+      <c r="M10" t="s">
+        <v>56</v>
+      </c>
+      <c r="P10" t="s">
+        <v>62</v>
+      </c>
+      <c r="R10" t="s">
+        <v>26</v>
+      </c>
+      <c r="S10" t="s">
+        <v>27</v>
+      </c>
+      <c r="T10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11" t="s">
+        <v>65</v>
+      </c>
+      <c r="M11" t="s">
+        <v>56</v>
+      </c>
+      <c r="P11" t="s">
+        <v>62</v>
+      </c>
+      <c r="R11" t="s">
+        <v>26</v>
+      </c>
+      <c r="S11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T11" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -750,7 +850,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -762,25 +862,25 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="F1" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="G1" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="H1" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I1" t="s">
         <v>12</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="K1" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
@@ -788,19 +888,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="E2" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="I2" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="J2" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3">
@@ -817,7 +917,7 @@
         <v>50</v>
       </c>
       <c r="H3" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="J3" t="s">
         <v>47</v>
@@ -828,19 +928,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="C4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E4" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="H4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="I4" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="J4" t="s">
         <v>47</v>
@@ -851,13 +951,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C5" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="E5" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="J5" t="s">
         <v>47</v>
@@ -872,7 +972,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -884,25 +984,28 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="F1" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="G1" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="H1" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I1" t="s">
-        <v>12</v>
+        <v>87</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="K1" t="s">
-        <v>65</v>
+        <v>88</v>
+      </c>
+      <c r="L1" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="2">
@@ -910,19 +1013,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="E2" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="H2" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="J2" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3">
@@ -930,16 +1033,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="C3" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E3" t="s">
-        <v>86</v>
+        <v>95</v>
+      </c>
+      <c r="H3" t="s">
+        <v>96</v>
+      </c>
+      <c r="I3" t="s">
+        <v>97</v>
       </c>
       <c r="J3" t="s">
         <v>47</v>
+      </c>
+      <c r="K3" s="1">
+        <v>44880</v>
       </c>
     </row>
     <row r="4">
@@ -947,19 +1059,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="E4" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="H4" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="J4" t="s">
         <v>47</v>
+      </c>
+      <c r="K4" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="5">
@@ -967,22 +1082,25 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="C5" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E5" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="H5" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="I5" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="J5" t="s">
         <v>47</v>
+      </c>
+      <c r="K5" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -994,7 +1112,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1006,25 +1124,25 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="F1" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="G1" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="H1" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I1" t="s">
         <v>12</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="K1" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
@@ -1032,19 +1150,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="E2" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="H2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="J2" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3">
@@ -1052,16 +1170,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="C3" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E3" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J3" t="s">
         <v>47</v>
@@ -1072,16 +1190,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="C4" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="E4" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="H4" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="J4" t="s">
         <v>47</v>
@@ -1096,10 +1214,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="B1" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -1108,16 +1226,16 @@
         <v>1</v>
       </c>
       <c r="E1" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="F1" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="G1" t="s">
         <v>12</v>
       </c>
       <c r="H1" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2">
@@ -1125,16 +1243,16 @@
         <v>44742</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="E2" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="F2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="H2" t="s">
         <v>47</v>
@@ -1145,19 +1263,19 @@
         <v>44972</v>
       </c>
       <c r="B3" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C3" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="D3" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="E3" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="F3" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="H3" t="s">
         <v>47</v>
@@ -1165,19 +1283,19 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="C4" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="D4" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="E4" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="F4" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="G4" t="s">
         <v>52</v>
@@ -1188,22 +1306,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="B5" s="1">
         <v>44119</v>
       </c>
       <c r="C5" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="D5" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E5" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="F5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H5" t="s">
         <v>47</v>
@@ -1211,16 +1329,16 @@
     </row>
     <row r="6">
       <c r="C6" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="D6" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="E6" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="F6" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="H6" t="s">
         <v>47</v>
@@ -1228,16 +1346,16 @@
     </row>
     <row r="7">
       <c r="C7" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="D7" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="E7" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="F7" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="H7" t="s">
         <v>47</v>
@@ -1245,19 +1363,19 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="C8" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="D8" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="E8" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="F8" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="H8" t="s">
         <v>47</v>
@@ -1268,10 +1386,10 @@
         <v>45047</v>
       </c>
       <c r="E9" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="F9" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="H9" t="s">
         <v>47</v>
@@ -1292,7 +1410,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="D1" t="s">
         <v>12</v>
@@ -1301,23 +1419,37 @@
         <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C2" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="D2" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="F2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" t="s">
+        <v>131</v>
+      </c>
+      <c r="F3" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1336,7 +1468,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="D1" t="s">
         <v>12</v>
@@ -1345,18 +1477,18 @@
         <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="F2" t="s">
         <v>47</v>

</xml_diff>